<commit_message>
feat: add WeLink CLI automation generator demo tool
</commit_message>
<xml_diff>
--- a/tools-platform/data/images/mpfftz2k_5.xlsx
+++ b/tools-platform/data/images/mpfftz2k_5.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="141">
   <si>
     <t>分组 (Group)</t>
   </si>
@@ -945,12 +945,8 @@
       </c>
     </row>
     <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2">
-        <v>34</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
@@ -989,12 +985,8 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2">
-        <v>34</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>29</v>
       </c>
@@ -1033,12 +1025,8 @@
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2">
-        <v>34</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
@@ -1077,12 +1065,8 @@
       </c>
     </row>
     <row r="6" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2">
-        <v>34</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>39</v>
       </c>
@@ -1121,12 +1105,8 @@
       </c>
     </row>
     <row r="7" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="2">
-        <v>34</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
         <v>45</v>
       </c>
@@ -1165,12 +1145,8 @@
       </c>
     </row>
     <row r="8" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="2">
-        <v>34</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
         <v>50</v>
       </c>
@@ -1209,12 +1185,8 @@
       </c>
     </row>
     <row r="9" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2">
-        <v>34</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
         <v>52</v>
       </c>
@@ -1253,12 +1225,8 @@
       </c>
     </row>
     <row r="10" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="2">
-        <v>34</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1297,12 +1265,8 @@
       </c>
     </row>
     <row r="11" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="2">
-        <v>34</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
         <v>61</v>
       </c>
@@ -1341,12 +1305,8 @@
       </c>
     </row>
     <row r="12" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="2">
-        <v>34</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
         <v>65</v>
       </c>
@@ -1429,12 +1389,8 @@
       </c>
     </row>
     <row r="14" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" s="2">
-        <v>16</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
       <c r="C14" s="2" t="s">
         <v>74</v>
       </c>
@@ -1473,12 +1429,8 @@
       </c>
     </row>
     <row r="15" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="2">
-        <v>16</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="2" t="s">
         <v>75</v>
       </c>
@@ -1517,12 +1469,8 @@
       </c>
     </row>
     <row r="16" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="2">
-        <v>16</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
         <v>76</v>
       </c>
@@ -1561,12 +1509,8 @@
       </c>
     </row>
     <row r="17" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="2">
-        <v>16</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
         <v>79</v>
       </c>
@@ -1605,12 +1549,8 @@
       </c>
     </row>
     <row r="18" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="2">
-        <v>16</v>
-      </c>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
       <c r="C18" s="2" t="s">
         <v>83</v>
       </c>
@@ -1649,12 +1589,8 @@
       </c>
     </row>
     <row r="19" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="2">
-        <v>16</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
         <v>85</v>
       </c>
@@ -1693,12 +1629,8 @@
       </c>
     </row>
     <row r="20" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="2">
-        <v>16</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
         <v>86</v>
       </c>
@@ -1781,12 +1713,8 @@
       </c>
     </row>
     <row r="22" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B22" s="2">
-        <v>10</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
       <c r="C22" s="2" t="s">
         <v>90</v>
       </c>
@@ -1825,12 +1753,8 @@
       </c>
     </row>
     <row r="23" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B23" s="2">
-        <v>10</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="2" t="s">
         <v>91</v>
       </c>
@@ -1869,12 +1793,8 @@
       </c>
     </row>
     <row r="24" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B24" s="2">
-        <v>10</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
         <v>93</v>
       </c>
@@ -1957,12 +1877,8 @@
       </c>
     </row>
     <row r="26" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B26" s="2">
-        <v>5</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
         <v>96</v>
       </c>
@@ -2001,12 +1917,8 @@
       </c>
     </row>
     <row r="27" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B27" s="2">
-        <v>5</v>
-      </c>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
         <v>97</v>
       </c>
@@ -2045,12 +1957,8 @@
       </c>
     </row>
     <row r="28" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B28" s="2">
-        <v>5</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
         <v>98</v>
       </c>
@@ -2089,12 +1997,8 @@
       </c>
     </row>
     <row r="29" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B29" s="2">
-        <v>5</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
         <v>99</v>
       </c>
@@ -2177,12 +2081,8 @@
       </c>
     </row>
     <row r="31" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B31" s="2">
-        <v>9</v>
-      </c>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
         <v>102</v>
       </c>
@@ -2221,12 +2121,8 @@
       </c>
     </row>
     <row r="32" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B32" s="2">
-        <v>9</v>
-      </c>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
         <v>103</v>
       </c>
@@ -2265,12 +2161,8 @@
       </c>
     </row>
     <row r="33" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B33" s="2">
-        <v>9</v>
-      </c>
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
       <c r="C33" s="2" t="s">
         <v>110</v>
       </c>
@@ -2309,12 +2201,8 @@
       </c>
     </row>
     <row r="34" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B34" s="2">
-        <v>9</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
       <c r="C34" s="2" t="s">
         <v>116</v>
       </c>
@@ -2353,12 +2241,8 @@
       </c>
     </row>
     <row r="35" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B35" s="2">
-        <v>9</v>
-      </c>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
         <v>122</v>
       </c>
@@ -2397,12 +2281,8 @@
       </c>
     </row>
     <row r="36" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B36" s="2">
-        <v>9</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
       <c r="C36" s="2" t="s">
         <v>123</v>
       </c>
@@ -2441,12 +2321,8 @@
       </c>
     </row>
     <row r="37" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B37" s="2">
-        <v>9</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
         <v>124</v>
       </c>
@@ -2485,12 +2361,8 @@
       </c>
     </row>
     <row r="38" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B38" s="2">
-        <v>9</v>
-      </c>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
       <c r="C38" s="2" t="s">
         <v>126</v>
       </c>
@@ -2573,12 +2445,8 @@
       </c>
     </row>
     <row r="40" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B40" s="2">
-        <v>10</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
       <c r="C40" s="2" t="s">
         <v>129</v>
       </c>
@@ -2749,12 +2617,8 @@
       </c>
     </row>
     <row r="44" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B44" s="2">
-        <v>40</v>
-      </c>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
       <c r="C44" s="2" t="s">
         <v>136</v>
       </c>
@@ -2793,12 +2657,8 @@
       </c>
     </row>
     <row r="45" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B45" s="2">
-        <v>40</v>
-      </c>
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
       <c r="C45" s="2" t="s">
         <v>137</v>
       </c>
@@ -2837,12 +2697,8 @@
       </c>
     </row>
     <row r="46" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B46" s="2">
-        <v>40</v>
-      </c>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
       <c r="C46" s="2" t="s">
         <v>138</v>
       </c>
@@ -2881,12 +2737,8 @@
       </c>
     </row>
     <row r="47" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B47" s="2">
-        <v>40</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
       <c r="C47" s="2" t="s">
         <v>139</v>
       </c>
@@ -2942,6 +2794,22 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="B2:B12"/>
+    <mergeCell ref="A13:A20"/>
+    <mergeCell ref="B13:B20"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="B25:B29"/>
+    <mergeCell ref="A30:A38"/>
+    <mergeCell ref="B30:B38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="A43:A47"/>
+    <mergeCell ref="B43:B47"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>